<commit_message>
test tri par chapitre
</commit_message>
<xml_diff>
--- a/convergence-export/src/main/resources/template-export-convergence.xlsx
+++ b/convergence-export/src/main/resources/template-export-convergence.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27231"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flabatie\Documents\ENV-ANS\19-PLUGIN-SQUASH\Claire2\squash-plugin\convergence-export\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B2E9D12-3485-44FF-A65A-B775DA7DE925}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A4C1372-6005-46B5-91D3-55B9D648A1F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14520" yWindow="-18120" windowWidth="29040" windowHeight="17790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="-16320" windowWidth="29040" windowHeight="15990" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exigences" sheetId="1" r:id="rId1"/>
+    <sheet name="Feuil1" sheetId="3" r:id="rId2"/>
+    <sheet name="ExigencesTriees" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">Exigences!$C$1:$J$1</definedName>
@@ -56,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="19">
   <si>
     <t>Profil</t>
   </si>
@@ -683,4 +685,72 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D626AE9-221F-4CB5-8618-E9799652F9CF}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="18.5"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C04B193-E64F-417A-AB13-9CA521A2130D}">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.2109375" defaultRowHeight="15.5"/>
+  <cols>
+    <col min="1" max="1" width="13.42578125" style="7" customWidth="1"/>
+    <col min="2" max="2" width="13.2109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="37.92578125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="35.2109375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="66.42578125" style="3" customWidth="1"/>
+    <col min="6" max="6" width="12.2109375" style="2" customWidth="1"/>
+    <col min="7" max="7" width="18.5703125" style="4" customWidth="1"/>
+    <col min="8" max="8" width="66.42578125" style="5" customWidth="1"/>
+    <col min="9" max="9" width="18.5703125" style="6" customWidth="1"/>
+    <col min="10" max="10" width="30.5703125" style="5" customWidth="1"/>
+    <col min="11" max="11" width="16.42578125" style="7" customWidth="1"/>
+    <col min="12" max="16384" width="9.2109375" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" s="1" customFormat="1" ht="56.25" customHeight="1">
+      <c r="A1" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" s="17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>